<commit_message>
Update reports, CSVs, and snapshots for no-date
</commit_message>
<xml_diff>
--- a/data/reports/2024-03-04/2024-03-04_duplicates.xlsx
+++ b/data/reports/2024-03-04/2024-03-04_duplicates.xlsx
@@ -140,7 +140,7 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=ff8966501bb7f810027562cae54bcb7f&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0004801</t>
+    <t>RMD0004807</t>
   </si>
   <si>
     <t>E-Vergent.Com LLC</t>
@@ -153,12 +153,6 @@
     <t>none</t>
   </si>
   <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=949115a61bc13c102eb2a82fe54bcb0c&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0004807</t>
-  </si>
-  <si>
     <t>Shawn Tarlo</t>
   </si>
   <si>
@@ -184,7 +178,13 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=470739ea1bc93c102eb2a82fe54bcba1&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0005143</t>
+    <t>RMD0004801</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=949115a61bc13c102eb2a82fe54bcb0c&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0004495</t>
   </si>
   <si>
     <t>Ooma, Inc.</t>
@@ -195,6 +195,30 @@
 SUNNYVALE CA 94085</t>
   </si>
   <si>
+    <t>0023473408; 0025715012; 0028440600; 0021330824; 0022722623</t>
+  </si>
+  <si>
+    <t>Tobin Farrand</t>
+  </si>
+  <si>
+    <t>Vice President, Engineering &amp; Operations</t>
+  </si>
+  <si>
+    <t>Engineering &amp; Operations</t>
+  </si>
+  <si>
+    <t>6505666600</t>
+  </si>
+  <si>
+    <t>2024-02-26</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=cff38bf91b05f4109294113d9c4bcb69&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0005143</t>
+  </si>
+  <si>
     <t>0023473408
 0025715012
 0028440600</t>
@@ -213,31 +237,7 @@
 SUNNYVALE CA 94085</t>
   </si>
   <si>
-    <t>6505666600</t>
-  </si>
-  <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=b165a0c21b0e3410503110ad9c4bcbce&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0004495</t>
-  </si>
-  <si>
-    <t>0023473408; 0025715012; 0028440600; 0021330824; 0022722623</t>
-  </si>
-  <si>
-    <t>Tobin Farrand</t>
-  </si>
-  <si>
-    <t>Vice President, Engineering &amp; Operations</t>
-  </si>
-  <si>
-    <t>Engineering &amp; Operations</t>
-  </si>
-  <si>
-    <t>2024-02-26</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=cff38bf91b05f4109294113d9c4bcb69&amp;view=sp</t>
   </si>
   <si>
     <t>RMD0005813</t>
@@ -280,7 +280,7 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=0df870c21bcdf41002beea82f54bcba2&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0009352</t>
+    <t>RMD0004139</t>
   </si>
   <si>
     <t>Global Net Holdings, Inc.</t>
@@ -296,6 +296,21 @@
     <t>CEO</t>
   </si>
   <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>800-709-6314</t>
+  </si>
+  <si>
+    <t>2022-09-15</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=c77b62251b09741002beea82f54bcb87&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0009352</t>
+  </si>
+  <si>
     <t>Financial</t>
   </si>
   <si>
@@ -306,21 +321,6 @@
   </si>
   <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=b379943f1be37810cc2f2f82f54bcbf5&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0004139</t>
-  </si>
-  <si>
-    <t>Sales</t>
-  </si>
-  <si>
-    <t>800-709-6314</t>
-  </si>
-  <si>
-    <t>2022-09-15</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=c77b62251b09741002beea82f54bcb87&amp;view=sp</t>
   </si>
   <si>
     <t>RMD0008972</t>
@@ -430,7 +430,7 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=53ad1e731b53b0109294113d9c4bcb6a&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0006774</t>
+    <t>RMD0008869</t>
   </si>
   <si>
     <t>Sage Communications, Inc.</t>
@@ -440,40 +440,40 @@
 Camarillo CA 93012</t>
   </si>
   <si>
+    <t>Sage Network &amp; Communications</t>
+  </si>
+  <si>
+    <t>Rick Minyard</t>
+  </si>
+  <si>
+    <t>Officer</t>
+  </si>
+  <si>
+    <t>Exec</t>
+  </si>
+  <si>
+    <t>8059141801</t>
+  </si>
+  <si>
+    <t>1855</t>
+  </si>
+  <si>
+    <t>2024-02-02</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=ed3d8a531b0334509ac2ea04bc4bcb27&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0006774</t>
+  </si>
+  <si>
     <t>NONE</t>
   </si>
   <si>
-    <t>Sage Network &amp; Communications</t>
-  </si>
-  <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=612a08851bbef010e1ca848ce54bcbb3&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0008869</t>
-  </si>
-  <si>
-    <t>Rick Minyard</t>
-  </si>
-  <si>
-    <t>Officer</t>
-  </si>
-  <si>
-    <t>Exec</t>
-  </si>
-  <si>
-    <t>8059141801</t>
-  </si>
-  <si>
-    <t>1855</t>
-  </si>
-  <si>
-    <t>2024-02-02</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=ed3d8a531b0334509ac2ea04bc4bcb27&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0003929</t>
+    <t>RMD0004389</t>
   </si>
   <si>
     <t>Idealtel Dominicana USA, Inc. dba myidealtel.com</t>
@@ -484,16 +484,16 @@
 Cooper City FL 33328</t>
   </si>
   <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=9a075a791b8db4109294113d9c4bcbd5&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0003929</t>
+  </si>
+  <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=fab855e51b09741064c4426de54bcbf6&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0004389</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=9a075a791b8db4109294113d9c4bcbd5&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0005819</t>
+    <t>RMD0004724</t>
   </si>
   <si>
     <t>Ton80 Communications, LLC</t>
@@ -503,16 +503,16 @@
 Anderson SC 29642</t>
   </si>
   <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=6239f4c21bcdf41002beea82f54bcb2a&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0005819</t>
+  </si>
+  <si>
     <t>4109121000</t>
   </si>
   <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=aab7f5961b667c10dabd2f41f54bcb9f&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0004724</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=6239f4c21bcdf41002beea82f54bcb2a&amp;view=sp</t>
   </si>
   <si>
     <t>RMD0004806</t>
@@ -553,10 +553,20 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=beda02fb1bc5f05064c4426de54bcb94&amp;view=sp</t>
   </si>
   <si>
+    <t>RMD0005785</t>
+  </si>
+  <si>
+    <t>Edge Fibernet</t>
+  </si>
+  <si>
+    <t>5004 4th Avenue
+Brooklyn New York 11220</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=5dcfb14e1bea3c105e240f6fe54bcb62&amp;view=sp</t>
+  </si>
+  <si>
     <t>RMD0005786</t>
-  </si>
-  <si>
-    <t>Edge Fibernet</t>
   </si>
   <si>
     <t>254 36th Street
@@ -567,20 +577,33 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=eb20864e1bea3c105e240f6fe54bcbf1&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0005785</t>
-  </si>
-  <si>
-    <t>5004 4th Avenue
-Brooklyn New York 11220</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=5dcfb14e1bea3c105e240f6fe54bcb62&amp;view=sp</t>
+    <t>RMD0003758</t>
+  </si>
+  <si>
+    <t>Matchcom Telecommunications Inc.</t>
+  </si>
+  <si>
+    <t>1680 Michigan Ave
+Ste 700
+Miami Beach Florida 33139</t>
+  </si>
+  <si>
+    <t>Davon Person</t>
+  </si>
+  <si>
+    <t>Director of Operations</t>
+  </si>
+  <si>
+    <t>Network Operations Center</t>
+  </si>
+  <si>
+    <t>9546248162</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=494bb99d1bcdf0109294113d9c4bcb26&amp;view=sp</t>
   </si>
   <si>
     <t>RMD0007488</t>
-  </si>
-  <si>
-    <t>Matchcom Telecommunications Inc.</t>
   </si>
   <si>
     <t>1680 Michigan Ave
@@ -614,33 +637,30 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=267cc9661b3ef410aa3cea41f54bcbcd&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0003758</t>
-  </si>
-  <si>
-    <t>1680 Michigan Ave
-Ste 700
-Miami Beach Florida 33139</t>
-  </si>
-  <si>
-    <t>Davon Person</t>
-  </si>
-  <si>
-    <t>Director of Operations</t>
-  </si>
-  <si>
-    <t>Network Operations Center</t>
-  </si>
-  <si>
-    <t>9546248162</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=494bb99d1bcdf0109294113d9c4bcb26&amp;view=sp</t>
+    <t>RMD0008297</t>
+  </si>
+  <si>
+    <t>GloTell US Corp.</t>
+  </si>
+  <si>
+    <t>1830 S Ocean Drive
+Suite 902
+Halladale Beach FL 33009</t>
+  </si>
+  <si>
+    <t>Alina Karpova</t>
+  </si>
+  <si>
+    <t>Administration</t>
+  </si>
+  <si>
+    <t>9548354110</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=ffdd33cb1bfe781093d3a820f54bcb29&amp;view=sp</t>
   </si>
   <si>
     <t>RMD0002900</t>
-  </si>
-  <si>
-    <t>GloTell US Corp.</t>
   </si>
   <si>
     <t>1001 North Federal Hwy
@@ -667,26 +687,6 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=0a82aeaf1b7430507ccf20ecac4bcb54&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0008297</t>
-  </si>
-  <si>
-    <t>1830 S Ocean Drive
-Suite 902
-Halladale Beach FL 33009</t>
-  </si>
-  <si>
-    <t>Alina Karpova</t>
-  </si>
-  <si>
-    <t>Administration</t>
-  </si>
-  <si>
-    <t>9548354110</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=ffdd33cb1bfe781093d3a820f54bcb29&amp;view=sp</t>
-  </si>
-  <si>
     <t>RMD0009294</t>
   </si>
   <si>
@@ -763,7 +763,7 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=64046a611bc1b4102eb2a82fe54bcb32&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0005124</t>
+    <t>RMD0005139</t>
   </si>
   <si>
     <t>Opentact Inc</t>
@@ -774,12 +774,6 @@
 Cheyenne WY 82009</t>
   </si>
   <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=f40ce7d11b8eb01068d1a82eac4bcbde&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0005139</t>
-  </si>
-  <si>
     <t>Anne Kwong</t>
   </si>
   <si>
@@ -802,6 +796,12 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=89cc84f51b4af01068d1a82eac4bcb3e&amp;view=sp</t>
   </si>
   <si>
+    <t>RMD0005124</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=f40ce7d11b8eb01068d1a82eac4bcbde&amp;view=sp</t>
+  </si>
+  <si>
     <t>RMD0004701</t>
   </si>
   <si>
@@ -845,7 +845,7 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=296153731b30b0507ccf20ecac4bcbd8&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0003053</t>
+    <t>RMD0009640</t>
   </si>
   <si>
     <t>The Kalson Inc Limited</t>
@@ -855,22 +855,22 @@
  UB10 0AD UXBRIDGE, United Kingdom</t>
   </si>
   <si>
+    <t>Anum Rasheed Kalson</t>
+  </si>
+  <si>
+    <t>'+92-3222100249</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=1e7857331b4885103e8aa93be54bcb79&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0003053</t>
+  </si>
+  <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=73375fbb1b30b0507ccf20ecac4bcb1c&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0009640</t>
-  </si>
-  <si>
-    <t>Anum Rasheed Kalson</t>
-  </si>
-  <si>
-    <t>'+92-3222100249</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=1e7857331b4885103e8aa93be54bcb79&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0003442</t>
+    <t>RMD0003444</t>
   </si>
   <si>
     <t>Shaw Telecom GP</t>
@@ -881,6 +881,32 @@
   </si>
   <si>
     <t>Canada</t>
+  </si>
+  <si>
+    <t>0031064868; 0031064884; 0031064900</t>
+  </si>
+  <si>
+    <t>SHAW CORP; 1503357 Alberta Ltd.; 1950036 Ontario Ltd.; Mid-Bowline Group Corp.; Mid-Bowline Holdings Corp.; Wind Mobile Corp.; Freedom Mobile Inc.</t>
+  </si>
+  <si>
+    <t>Network Operations</t>
+  </si>
+  <si>
+    <t>TOPS-NR&amp;A</t>
+  </si>
+  <si>
+    <t>2728 Hopewell Place N.E.
+Calgary AE 17724
+Alberta</t>
+  </si>
+  <si>
+    <t>'+1-866-244-7475</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=5d9f0e581b8df0509294113d9c4bcb95&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0003442</t>
   </si>
   <si>
     <t>0031064868;
@@ -900,33 +926,7 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=322c4e941b8df0509294113d9c4bcb51&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0003444</t>
-  </si>
-  <si>
-    <t>0031064868; 0031064884; 0031064900</t>
-  </si>
-  <si>
-    <t>SHAW CORP; 1503357 Alberta Ltd.; 1950036 Ontario Ltd.; Mid-Bowline Group Corp.; Mid-Bowline Holdings Corp.; Wind Mobile Corp.; Freedom Mobile Inc.</t>
-  </si>
-  <si>
-    <t>Network Operations</t>
-  </si>
-  <si>
-    <t>TOPS-NR&amp;A</t>
-  </si>
-  <si>
-    <t>2728 Hopewell Place N.E.
-Calgary AE 17724
-Alberta</t>
-  </si>
-  <si>
-    <t>'+1-866-244-7475</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=5d9f0e581b8df0509294113d9c4bcb95&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0007384</t>
+    <t>RMD0003705</t>
   </si>
   <si>
     <t>Axkan Consultores S. de R.L. de C.V.</t>
@@ -939,6 +939,12 @@
     <t>Mexico</t>
   </si>
   <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=76af51511bc9f0102eb2a82fe54bcb18&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0007384</t>
+  </si>
+  <si>
     <t>Juan Carlos Bravo Abarca</t>
   </si>
   <si>
@@ -946,12 +952,6 @@
   </si>
   <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=47035e5e1b7eb4109ac2ea04bc4bcbb1&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0003705</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=76af51511bc9f0102eb2a82fe54bcb18&amp;view=sp</t>
   </si>
   <si>
     <t>RMD0009817</t>
@@ -1061,7 +1061,7 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=93ebdbd01b227810ca5aec21f54bcbd6&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0005297</t>
+    <t>RMD0007936</t>
   </si>
   <si>
     <t>STREAMLINE SELLERS PTY LTD</t>
@@ -1074,22 +1074,22 @@
     <t>Australia</t>
   </si>
   <si>
+    <t>Syed Omar Farooq Shah</t>
+  </si>
+  <si>
+    <t>'+61406851546</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=6273a2321b3638109ac2ea04bc4bcb55&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0005297</t>
+  </si>
+  <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=d24a9a271bca3810d49ca86ce54bcb20&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0007936</t>
-  </si>
-  <si>
-    <t>Syed Omar Farooq Shah</t>
-  </si>
-  <si>
-    <t>'+61406851546</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=6273a2321b3638109ac2ea04bc4bcb55&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0005585</t>
+    <t>RMD0005574</t>
   </si>
   <si>
     <t>MegaClec, Inc</t>
@@ -1103,6 +1103,18 @@
     <t>0012465480</t>
   </si>
   <si>
+    <t>Troy City Internet Exchange;Voiceway;Meganet Communications</t>
+  </si>
+  <si>
+    <t>5086460030</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=1426e7581ba678109294113d9c4bcb2f&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0005585</t>
+  </si>
+  <si>
     <t>Voiceay, Voiceway Netoworks, Meganet,  Troy City Internet Exchange</t>
   </si>
   <si>
@@ -1116,19 +1128,29 @@
 Fall River MA 02721</t>
   </si>
   <si>
-    <t>5086460030</t>
-  </si>
-  <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=c9f5735c1ba2781002beea82f54bcbaf&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0005574</t>
-  </si>
-  <si>
-    <t>Troy City Internet Exchange;Voiceway;Meganet Communications</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=1426e7581ba678109294113d9c4bcb2f&amp;view=sp</t>
+    <t>RMD0007962</t>
+  </si>
+  <si>
+    <t>office no 17 3rd floor anique arcade pla
+federal 46000 Islamabad, Pakistan</t>
+  </si>
+  <si>
+    <t>Pakistan</t>
+  </si>
+  <si>
+    <t>Umair Hassan</t>
+  </si>
+  <si>
+    <t>Executive</t>
+  </si>
+  <si>
+    <t>'+92-333-6778-636</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=8037e23e1b32781093d3a820f54bcb1c&amp;view=sp</t>
   </si>
   <si>
     <t>RMD0006284</t>
@@ -1138,29 +1160,7 @@
   Islamabad, Pakistan</t>
   </si>
   <si>
-    <t>Pakistan</t>
-  </si>
-  <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=3acc71c31b2a305064c4426de54bcb40&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0007962</t>
-  </si>
-  <si>
-    <t>office no 17 3rd floor anique arcade pla
-federal 46000 Islamabad, Pakistan</t>
-  </si>
-  <si>
-    <t>Umair Hassan</t>
-  </si>
-  <si>
-    <t>Executive</t>
-  </si>
-  <si>
-    <t>'+92-333-6778-636</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=8037e23e1b32781093d3a820f54bcb1c&amp;view=sp</t>
   </si>
   <si>
     <t>RMD0008125</t>
@@ -1192,7 +1192,7 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=3cc1fbbe1b7a3810dcd1ed3be54bcbe8&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0007575</t>
+    <t>RMD0007626</t>
   </si>
   <si>
     <t>Turcios Parada SA</t>
@@ -1205,16 +1205,16 @@
     <t>El Salvador</t>
   </si>
   <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=5b6a75a61b3af410680f657ae54bcbbd&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0007575</t>
+  </si>
+  <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=cfeb296a1bf6f410680f657ae54bcbeb&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0007626</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=5b6a75a61b3af410680f657ae54bcbbd&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0007696</t>
+    <t>RMD0007716</t>
   </si>
   <si>
     <t>High Country Internet</t>
@@ -1224,16 +1224,16 @@
 Tucson AZ 85719</t>
   </si>
   <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=4a516ea21b7ef410165aedfde54bcbd3&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0007696</t>
+  </si>
+  <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=e3d356aa1b3ef410165aedfde54bcb51&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0007716</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=4a516ea21b7ef410165aedfde54bcbd3&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0007944</t>
+    <t>RMD0007939</t>
   </si>
   <si>
     <t>Conquest Solutions</t>
@@ -1243,6 +1243,12 @@
 Marietta GA 30067</t>
   </si>
   <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=d225a2fe1b7a3810e4ccdb1de54bcbff&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0007944</t>
+  </si>
+  <si>
     <t>Lance Retter</t>
   </si>
   <si>
@@ -1255,13 +1261,7 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=c186e6321bba3810e4ccdb1de54bcb5a&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0007939</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=d225a2fe1b7a3810e4ccdb1de54bcbff&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0008097</t>
+    <t>RMD0008064</t>
   </si>
   <si>
     <t>Sam Asher Computing Services, Inc.</t>
@@ -1276,6 +1276,12 @@
 Hyper-Reach</t>
   </si>
   <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=39639b3a1b3a3810dcd1ed3be54bcb5e&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0008097</t>
+  </si>
+  <si>
     <t>Caitlin Olfano</t>
   </si>
   <si>
@@ -1288,13 +1294,7 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=4172e7f21b7a3810dcd1ed3be54bcbb5&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0008064</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=39639b3a1b3a3810dcd1ed3be54bcb5e&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0008393</t>
+    <t>RMD0008423</t>
   </si>
   <si>
     <t>Your Business I.T. Inc.</t>
@@ -1302,12 +1302,6 @@
   <si>
     <t>295 Weber St. N
 Ontario N2J 3H8 Waterloo, Canada</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=545854ef1b7ab810d39dddb6bc4bcb74&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0008423</t>
   </si>
   <si>
     <t>Your Business I.T.</t>
@@ -1325,6 +1319,12 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=761bc9e71b3eb810d39dddb6bc4bcbe0&amp;view=sp</t>
   </si>
   <si>
+    <t>RMD0008393</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=545854ef1b7ab810d39dddb6bc4bcb74&amp;view=sp</t>
+  </si>
+  <si>
     <t>RMD0008451</t>
   </si>
   <si>
@@ -1344,7 +1344,7 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=b746a9e71bbeb81093d3a820f54bcb4c&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0008611</t>
+    <t>RMD0008612</t>
   </si>
   <si>
     <t>Liberty Wealth Planners</t>
@@ -1354,6 +1354,21 @@
  110065 Dehli, India</t>
   </si>
   <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Bharat Raj</t>
+  </si>
+  <si>
+    <t>'+919836963636</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=21f229c51b0bbc1093d3a820f54bcbdb&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0008611</t>
+  </si>
+  <si>
     <t>Bangladesh</t>
   </si>
   <si>
@@ -1369,44 +1384,29 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=9c9129851b0bbc1093d3a820f54bcb97&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0008612</t>
-  </si>
-  <si>
-    <t>India</t>
-  </si>
-  <si>
-    <t>Bharat Raj</t>
-  </si>
-  <si>
-    <t>'+919836963636</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=21f229c51b0bbc1093d3a820f54bcbdb&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0008756</t>
+    <t>RMD0008759</t>
   </si>
   <si>
     <t>573 Ocean Blvd
 Hampton NH 03842</t>
   </si>
   <si>
+    <t>Jeffrey D Houston</t>
+  </si>
+  <si>
+    <t>6039294272</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=46724d021b0b3050003c43f1f54bcb05&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0008756</t>
+  </si>
+  <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=9bf181421b0b3050003c43f1f54bcbe8&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0008759</t>
-  </si>
-  <si>
-    <t>Jeffrey D Houston</t>
-  </si>
-  <si>
-    <t>6039294272</t>
-  </si>
-  <si>
-    <t>100</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=46724d021b0b3050003c43f1f54bcb05&amp;view=sp</t>
   </si>
   <si>
     <t>RMD0008755</t>
@@ -1473,7 +1473,7 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=3752aec61b0f3050003c43f1f54bcb54&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0009160</t>
+    <t>RMD0009161</t>
   </si>
   <si>
     <t>MCE Systems</t>
@@ -1483,16 +1483,16 @@
 Irvine CA 92604</t>
   </si>
   <si>
+    <t>9497014500</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=2338b76a1b577410503110ad9c4bcb43&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0009160</t>
+  </si>
+  <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=8975f3e61b577410503110ad9c4bcbcf&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0009161</t>
-  </si>
-  <si>
-    <t>9497014500</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=2338b76a1b577410503110ad9c4bcb43&amp;view=sp</t>
   </si>
   <si>
     <t>RMD0009453</t>
@@ -1527,7 +1527,7 @@
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=af63c18f1b3bb010c8e0ed3ce54bcb41&amp;view=sp</t>
   </si>
   <si>
-    <t>RMD0009728</t>
+    <t>RMD0009729</t>
   </si>
   <si>
     <t>Huffman Telcom Corp</t>
@@ -1537,22 +1537,22 @@
 Fort Collins CO 80524</t>
   </si>
   <si>
+    <t>Charlie Huffman</t>
+  </si>
+  <si>
+    <t>Customer Services</t>
+  </si>
+  <si>
+    <t>'+13033140978</t>
+  </si>
+  <si>
+    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=5dfd83771bac051085edebdbac4bcb2f&amp;view=sp</t>
+  </si>
+  <si>
+    <t>RMD0009728</t>
+  </si>
+  <si>
     <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=a48d8f371bac051085edebdbac4bcbba&amp;view=sp</t>
-  </si>
-  <si>
-    <t>RMD0009729</t>
-  </si>
-  <si>
-    <t>Charlie Huffman</t>
-  </si>
-  <si>
-    <t>Customer Services</t>
-  </si>
-  <si>
-    <t>'+13033140978</t>
-  </si>
-  <si>
-    <t>https://fccprod.servicenowservices.com/rmd?id=rmd_form&amp;table=x_g_fmc_rmd_robocall_mitigation_database&amp;sys_id=5dfd83771bac051085edebdbac4bcb2f&amp;view=sp</t>
   </si>
   <si>
     <t>RMD0012707</t>
@@ -6012,31 +6012,47 @@
       <c r="I5" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
+      <c r="J5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="P5" s="1"/>
-      <c r="Q5" s="1"/>
+      <c r="Q5" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="R5" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S5" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="U5" s="1"/>
+        <v>29</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>50</v>
+      </c>
       <c r="V5" s="1" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:22">
       <c r="A6" s="1" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="B6" s="1">
         <v>16082927</v>
@@ -6062,40 +6078,24 @@
       <c r="I6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>50</v>
-      </c>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
       <c r="P6" s="1"/>
-      <c r="Q6" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="Q6" s="1"/>
       <c r="R6" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S6" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>52</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="U6" s="1"/>
       <c r="V6" s="1" t="s">
         <v>53</v>
       </c>
@@ -6133,29 +6133,29 @@
       <c r="L7" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="M7" s="1"/>
+      <c r="N7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O7" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="P7" s="1"/>
       <c r="Q7" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S7" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="U7" s="1"/>
+        <v>26</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>62</v>
+      </c>
       <c r="V7" s="1" t="s">
         <v>63</v>
       </c>
@@ -6193,29 +6193,29 @@
       <c r="L8" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="M8" s="1"/>
+      <c r="M8" s="1" t="s">
+        <v>69</v>
+      </c>
       <c r="N8" s="1" t="s">
         <v>33</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P8" s="1"/>
       <c r="Q8" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S8" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>69</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="U8" s="1"/>
       <c r="V8" s="1" t="s">
         <v>70</v>
       </c>
@@ -6349,15 +6349,9 @@
       <c r="F11" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>43</v>
-      </c>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
       <c r="J11" s="1" t="s">
         <v>87</v>
       </c>
@@ -6378,13 +6372,13 @@
       </c>
       <c r="P11" s="1"/>
       <c r="Q11" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="T11" s="1" t="s">
         <v>29</v>
@@ -6415,9 +6409,15 @@
       <c r="F12" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
+      <c r="G12" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="J12" s="1" t="s">
         <v>87</v>
       </c>
@@ -6438,13 +6438,13 @@
       </c>
       <c r="P12" s="1"/>
       <c r="Q12" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="T12" s="1" t="s">
         <v>29</v>
@@ -6791,38 +6791,54 @@
       <c r="F19" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="G19" s="1"/>
+      <c r="H19" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="I19" s="1"/>
+      <c r="J19" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="1"/>
-      <c r="Q19" s="1"/>
+      <c r="K19" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="L19" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="P19" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q19" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="R19" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S19" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T19" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="U19" s="1"/>
+        <v>29</v>
+      </c>
+      <c r="U19" s="1" t="s">
+        <v>140</v>
+      </c>
       <c r="V19" s="1" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
     </row>
     <row r="20" spans="1:22">
       <c r="A20" s="1" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B20" s="1">
         <v>23250467</v>
@@ -6839,47 +6855,31 @@
       <c r="F20" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G20" s="1"/>
+      <c r="G20" s="1" t="s">
+        <v>143</v>
+      </c>
       <c r="H20" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I20" s="1"/>
-      <c r="J20" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="K20" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="M20" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="N20" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O20" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="P20" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="Q20" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+      <c r="P20" s="1"/>
+      <c r="Q20" s="1"/>
       <c r="R20" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S20" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T20" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="U20" s="1" t="s">
-        <v>143</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="U20" s="1"/>
       <c r="V20" s="1" t="s">
         <v>144</v>
       </c>
@@ -6994,45 +6994,31 @@
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
-      <c r="J23" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="K23" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="L23" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="N23" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O23" s="1" t="s">
-        <v>154</v>
-      </c>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
       <c r="P23" s="1"/>
-      <c r="Q23" s="1" t="s">
-        <v>80</v>
-      </c>
+      <c r="Q23" s="1"/>
       <c r="R23" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S23" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T23" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U23" s="1"/>
       <c r="V23" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="24" spans="1:22">
       <c r="A24" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B24" s="1">
         <v>25462672</v>
@@ -7052,22 +7038,36 @@
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
-      <c r="K24" s="1"/>
-      <c r="L24" s="1"/>
-      <c r="M24" s="1"/>
-      <c r="N24" s="1"/>
-      <c r="O24" s="1"/>
+      <c r="J24" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="M24" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="N24" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>156</v>
+      </c>
       <c r="P24" s="1"/>
-      <c r="Q24" s="1"/>
+      <c r="Q24" s="1" t="s">
+        <v>80</v>
+      </c>
       <c r="R24" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S24" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T24" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U24" s="1"/>
       <c r="V24" s="1" t="s">
@@ -7299,40 +7299,34 @@
       <c r="L29" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="M29" s="1" t="s">
+      <c r="M29" s="1"/>
+      <c r="N29" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O29" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="N29" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O29" s="1" t="s">
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="R29" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S29" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="T29" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="U29" s="1"/>
+      <c r="V29" s="1" t="s">
         <v>184</v>
-      </c>
-      <c r="P29" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="Q29" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="R29" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="S29" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="T29" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="U29" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="V29" s="1" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="30" spans="1:22">
       <c r="A30" s="1" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B30" s="1">
         <v>27710730</v>
@@ -7341,7 +7335,7 @@
         <v>178</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>29</v>
@@ -7353,35 +7347,41 @@
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
       <c r="J30" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="M30" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="K30" s="1" t="s">
+      <c r="N30" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O30" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="L30" s="1" t="s">
+      <c r="P30" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O30" s="1" t="s">
+      <c r="Q30" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="R30" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="S30" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="T30" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="U30" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="P30" s="1"/>
-      <c r="Q30" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="R30" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="S30" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="T30" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="U30" s="1"/>
       <c r="V30" s="1" t="s">
         <v>194</v>
       </c>
@@ -7406,47 +7406,47 @@
         <v>33</v>
       </c>
       <c r="G31" s="1"/>
-      <c r="H31" s="1" t="s">
-        <v>198</v>
-      </c>
+      <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="L31" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="K31" s="1" t="s">
+      <c r="M31" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="N31" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O31" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="L31" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="N31" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O31" s="1" t="s">
-        <v>202</v>
-      </c>
       <c r="P31" s="1"/>
-      <c r="Q31" s="1"/>
+      <c r="Q31" s="1" t="s">
+        <v>80</v>
+      </c>
       <c r="R31" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S31" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T31" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U31" s="1"/>
       <c r="V31" s="1" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="32" spans="1:22">
       <c r="A32" s="1" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B32" s="1">
         <v>27967686</v>
@@ -7455,7 +7455,7 @@
         <v>196</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>29</v>
@@ -7464,19 +7464,21 @@
         <v>33</v>
       </c>
       <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
+      <c r="H32" s="1" t="s">
+        <v>204</v>
+      </c>
       <c r="I32" s="1"/>
       <c r="J32" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="K32" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="K32" s="1" t="s">
-        <v>88</v>
-      </c>
       <c r="L32" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M32" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="M32" s="1" t="s">
-        <v>205</v>
       </c>
       <c r="N32" s="1" t="s">
         <v>33</v>
@@ -7485,17 +7487,15 @@
         <v>208</v>
       </c>
       <c r="P32" s="1"/>
-      <c r="Q32" s="1" t="s">
-        <v>80</v>
-      </c>
+      <c r="Q32" s="1"/>
       <c r="R32" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S32" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T32" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U32" s="1"/>
       <c r="V32" s="1" t="s">
@@ -7586,7 +7586,7 @@
       </c>
       <c r="P34" s="1"/>
       <c r="Q34" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R34" s="1" t="s">
         <v>26</v>
@@ -7652,7 +7652,7 @@
       </c>
       <c r="P35" s="1"/>
       <c r="Q35" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R35" s="1" t="s">
         <v>26</v>
@@ -7748,31 +7748,47 @@
       <c r="I37" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J37" s="1"/>
-      <c r="K37" s="1"/>
-      <c r="L37" s="1"/>
-      <c r="M37" s="1"/>
-      <c r="N37" s="1"/>
-      <c r="O37" s="1"/>
+      <c r="J37" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="K37" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="M37" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="N37" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O37" s="1" t="s">
+        <v>240</v>
+      </c>
       <c r="P37" s="1"/>
-      <c r="Q37" s="1"/>
+      <c r="Q37" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="R37" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S37" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T37" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="U37" s="1"/>
+        <v>29</v>
+      </c>
+      <c r="U37" s="1" t="s">
+        <v>241</v>
+      </c>
       <c r="V37" s="1" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
     </row>
     <row r="38" spans="1:22">
       <c r="A38" s="1" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="B38" s="1">
         <v>30149645</v>
@@ -7798,40 +7814,24 @@
       <c r="I38" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J38" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="K38" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="L38" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="M38" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="N38" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O38" s="1" t="s">
-        <v>242</v>
-      </c>
+      <c r="J38" s="1"/>
+      <c r="K38" s="1"/>
+      <c r="L38" s="1"/>
+      <c r="M38" s="1"/>
+      <c r="N38" s="1"/>
+      <c r="O38" s="1"/>
       <c r="P38" s="1"/>
-      <c r="Q38" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="Q38" s="1"/>
       <c r="R38" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S38" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T38" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="U38" s="1" t="s">
-        <v>243</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="U38" s="1"/>
       <c r="V38" s="1" t="s">
         <v>244</v>
       </c>
@@ -7878,7 +7878,7 @@
       </c>
       <c r="P39" s="1"/>
       <c r="Q39" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R39" s="1" t="s">
         <v>26</v>
@@ -7916,13 +7916,13 @@
         <v>256</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="J40" s="1" t="s">
         <v>248</v>
@@ -7980,31 +7980,45 @@
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
-      <c r="J41" s="1"/>
-      <c r="K41" s="1"/>
-      <c r="L41" s="1"/>
-      <c r="M41" s="1"/>
-      <c r="N41" s="1"/>
-      <c r="O41" s="1"/>
+      <c r="J41" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="K41" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="L41" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="M41" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="N41" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="O41" s="1" t="s">
+        <v>263</v>
+      </c>
       <c r="P41" s="1"/>
-      <c r="Q41" s="1"/>
+      <c r="Q41" s="1" t="s">
+        <v>38</v>
+      </c>
       <c r="R41" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S41" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T41" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U41" s="1"/>
       <c r="V41" s="1" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="42" spans="1:22">
       <c r="A42" s="1" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B42" s="1">
         <v>31063506</v>
@@ -8024,36 +8038,22 @@
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
-      <c r="J42" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="K42" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="L42" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="M42" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="N42" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="O42" s="1" t="s">
-        <v>265</v>
-      </c>
+      <c r="J42" s="1"/>
+      <c r="K42" s="1"/>
+      <c r="L42" s="1"/>
+      <c r="M42" s="1"/>
+      <c r="N42" s="1"/>
+      <c r="O42" s="1"/>
       <c r="P42" s="1"/>
-      <c r="Q42" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="Q42" s="1"/>
       <c r="R42" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S42" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T42" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U42" s="1"/>
       <c r="V42" s="1" t="s">
@@ -8086,31 +8086,45 @@
       <c r="I43" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="J43" s="1"/>
-      <c r="K43" s="1"/>
-      <c r="L43" s="1"/>
-      <c r="M43" s="1"/>
-      <c r="N43" s="1"/>
-      <c r="O43" s="1"/>
+      <c r="J43" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="K43" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="L43" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="M43" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="N43" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="O43" s="1" t="s">
+        <v>276</v>
+      </c>
       <c r="P43" s="1"/>
-      <c r="Q43" s="1"/>
+      <c r="Q43" s="1" t="s">
+        <v>38</v>
+      </c>
       <c r="R43" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S43" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T43" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U43" s="1"/>
       <c r="V43" s="1" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="44" spans="1:22">
       <c r="A44" s="1" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B44" s="1">
         <v>31064850</v>
@@ -8128,42 +8142,28 @@
         <v>270</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="H44" s="1"/>
       <c r="I44" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="J44" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="K44" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="L44" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="M44" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="N44" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="O44" s="1" t="s">
         <v>280</v>
       </c>
+      <c r="J44" s="1"/>
+      <c r="K44" s="1"/>
+      <c r="L44" s="1"/>
+      <c r="M44" s="1"/>
+      <c r="N44" s="1"/>
+      <c r="O44" s="1"/>
       <c r="P44" s="1"/>
-      <c r="Q44" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="Q44" s="1"/>
       <c r="R44" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S44" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T44" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U44" s="1"/>
       <c r="V44" s="1" t="s">
@@ -8192,45 +8192,31 @@
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
-      <c r="J45" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="K45" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="L45" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="M45" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="N45" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="O45" s="1" t="s">
-        <v>287</v>
-      </c>
+      <c r="J45" s="1"/>
+      <c r="K45" s="1"/>
+      <c r="L45" s="1"/>
+      <c r="M45" s="1"/>
+      <c r="N45" s="1"/>
+      <c r="O45" s="1"/>
       <c r="P45" s="1"/>
-      <c r="Q45" s="1" t="s">
-        <v>80</v>
-      </c>
+      <c r="Q45" s="1"/>
       <c r="R45" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S45" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T45" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U45" s="1"/>
       <c r="V45" s="1" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="46" spans="1:22">
       <c r="A46" s="1" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B46" s="1">
         <v>31092349</v>
@@ -8250,22 +8236,36 @@
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
-      <c r="J46" s="1"/>
-      <c r="K46" s="1"/>
-      <c r="L46" s="1"/>
-      <c r="M46" s="1"/>
-      <c r="N46" s="1"/>
-      <c r="O46" s="1"/>
+      <c r="J46" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="M46" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="N46" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="O46" s="1" t="s">
+        <v>289</v>
+      </c>
       <c r="P46" s="1"/>
-      <c r="Q46" s="1"/>
+      <c r="Q46" s="1" t="s">
+        <v>80</v>
+      </c>
       <c r="R46" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S46" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T46" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U46" s="1"/>
       <c r="V46" s="1" t="s">
@@ -8526,7 +8526,7 @@
       </c>
       <c r="P51" s="1"/>
       <c r="Q51" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R51" s="1" t="s">
         <v>26</v>
@@ -8620,31 +8620,45 @@
       <c r="G53" s="1"/>
       <c r="H53" s="1"/>
       <c r="I53" s="1"/>
-      <c r="J53" s="1"/>
-      <c r="K53" s="1"/>
-      <c r="L53" s="1"/>
-      <c r="M53" s="1"/>
-      <c r="N53" s="1"/>
-      <c r="O53" s="1"/>
+      <c r="J53" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="K53" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="L53" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="M53" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="N53" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="O53" s="1" t="s">
+        <v>330</v>
+      </c>
       <c r="P53" s="1"/>
-      <c r="Q53" s="1"/>
+      <c r="Q53" s="1" t="s">
+        <v>38</v>
+      </c>
       <c r="R53" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S53" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T53" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U53" s="1"/>
       <c r="V53" s="1" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="54" spans="1:22">
       <c r="A54" s="1" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B54" s="1">
         <v>31294614</v>
@@ -8664,36 +8678,22 @@
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
       <c r="I54" s="1"/>
-      <c r="J54" s="1" t="s">
-        <v>331</v>
-      </c>
-      <c r="K54" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="L54" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="M54" s="1" t="s">
-        <v>327</v>
-      </c>
-      <c r="N54" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="O54" s="1" t="s">
-        <v>332</v>
-      </c>
+      <c r="J54" s="1"/>
+      <c r="K54" s="1"/>
+      <c r="L54" s="1"/>
+      <c r="M54" s="1"/>
+      <c r="N54" s="1"/>
+      <c r="O54" s="1"/>
       <c r="P54" s="1"/>
-      <c r="Q54" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="Q54" s="1"/>
       <c r="R54" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S54" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T54" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U54" s="1"/>
       <c r="V54" s="1" t="s">
@@ -8725,46 +8725,40 @@
       <c r="H55" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="I55" s="1"/>
-      <c r="J55" s="1" t="s">
+      <c r="I55" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="J55" s="1"/>
+      <c r="K55" s="1"/>
+      <c r="L55" s="1"/>
+      <c r="M55" s="1"/>
+      <c r="N55" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O55" s="1" t="s">
         <v>339</v>
-      </c>
-      <c r="K55" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="L55" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="M55" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="N55" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O55" s="1" t="s">
-        <v>342</v>
       </c>
       <c r="P55" s="1"/>
       <c r="Q55" s="1" t="s">
         <v>38</v>
       </c>
       <c r="R55" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S55" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T55" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U55" s="1"/>
       <c r="V55" s="1" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
     <row r="56" spans="1:22">
       <c r="A56" s="1" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="B56" s="1">
         <v>31356652</v>
@@ -8785,33 +8779,39 @@
         <v>337</v>
       </c>
       <c r="H56" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="I56" s="1"/>
+      <c r="J56" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="K56" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="L56" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="M56" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="I56" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="J56" s="1"/>
-      <c r="K56" s="1"/>
-      <c r="L56" s="1"/>
-      <c r="M56" s="1"/>
       <c r="N56" s="1" t="s">
         <v>33</v>
       </c>
       <c r="O56" s="1" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="P56" s="1"/>
       <c r="Q56" s="1" t="s">
         <v>38</v>
       </c>
       <c r="R56" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S56" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T56" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U56" s="1"/>
       <c r="V56" s="1" t="s">
@@ -8835,47 +8835,55 @@
       <c r="F57" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="G57" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H57" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="I57" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="J57" s="1"/>
-      <c r="K57" s="1"/>
-      <c r="L57" s="1"/>
-      <c r="M57" s="1"/>
-      <c r="N57" s="1"/>
-      <c r="O57" s="1"/>
+      <c r="G57" s="1"/>
+      <c r="H57" s="1"/>
+      <c r="I57" s="1"/>
+      <c r="J57" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="K57" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="L57" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="M57" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="N57" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="O57" s="1" t="s">
+        <v>352</v>
+      </c>
       <c r="P57" s="1"/>
-      <c r="Q57" s="1"/>
+      <c r="Q57" s="1" t="s">
+        <v>38</v>
+      </c>
       <c r="R57" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S57" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T57" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U57" s="1"/>
       <c r="V57" s="1" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
     <row r="58" spans="1:22">
       <c r="A58" s="1" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B58" s="1">
         <v>31392434</v>
       </c>
       <c r="C58" s="1"/>
       <c r="D58" s="1" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>26</v>
@@ -8883,39 +8891,31 @@
       <c r="F58" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="G58" s="1"/>
-      <c r="H58" s="1"/>
-      <c r="I58" s="1"/>
-      <c r="J58" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="K58" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="L58" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="M58" s="1" t="s">
-        <v>352</v>
-      </c>
-      <c r="N58" s="1" t="s">
-        <v>349</v>
-      </c>
-      <c r="O58" s="1" t="s">
-        <v>355</v>
-      </c>
+      <c r="G58" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I58" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J58" s="1"/>
+      <c r="K58" s="1"/>
+      <c r="L58" s="1"/>
+      <c r="M58" s="1"/>
+      <c r="N58" s="1"/>
+      <c r="O58" s="1"/>
       <c r="P58" s="1"/>
-      <c r="Q58" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="Q58" s="1"/>
       <c r="R58" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S58" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T58" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U58" s="1"/>
       <c r="V58" s="1" t="s">
@@ -8951,7 +8951,7 @@
         <v>361</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="M59" s="1" t="s">
         <v>359</v>
@@ -8963,10 +8963,10 @@
         <v>362</v>
       </c>
       <c r="P59" s="1" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="Q59" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R59" s="1" t="s">
         <v>26</v>
@@ -9133,9 +9133,15 @@
       <c r="F63" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G63" s="1"/>
-      <c r="H63" s="1"/>
-      <c r="I63" s="1"/>
+      <c r="G63" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I63" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="J63" s="1"/>
       <c r="K63" s="1"/>
       <c r="L63" s="1"/>
@@ -9177,15 +9183,9 @@
       <c r="F64" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G64" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H64" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="I64" s="1" t="s">
-        <v>43</v>
-      </c>
+      <c r="G64" s="1"/>
+      <c r="H64" s="1"/>
+      <c r="I64" s="1"/>
       <c r="J64" s="1"/>
       <c r="K64" s="1"/>
       <c r="L64" s="1"/>
@@ -9222,55 +9222,39 @@
         <v>381</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="G65" s="1"/>
       <c r="H65" s="1"/>
       <c r="I65" s="1"/>
-      <c r="J65" s="1" t="s">
-        <v>382</v>
-      </c>
-      <c r="K65" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="L65" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="M65" s="1" t="s">
-        <v>381</v>
-      </c>
-      <c r="N65" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O65" s="1" t="s">
-        <v>383</v>
-      </c>
-      <c r="P65" s="1" t="s">
-        <v>384</v>
-      </c>
-      <c r="Q65" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="J65" s="1"/>
+      <c r="K65" s="1"/>
+      <c r="L65" s="1"/>
+      <c r="M65" s="1"/>
+      <c r="N65" s="1"/>
+      <c r="O65" s="1"/>
+      <c r="P65" s="1"/>
+      <c r="Q65" s="1"/>
       <c r="R65" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S65" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T65" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U65" s="1"/>
       <c r="V65" s="1" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="66" spans="1:22">
       <c r="A66" s="1" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="B66" s="1">
         <v>31445216</v>
@@ -9282,30 +9266,46 @@
         <v>381</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="G66" s="1"/>
       <c r="H66" s="1"/>
       <c r="I66" s="1"/>
-      <c r="J66" s="1"/>
-      <c r="K66" s="1"/>
-      <c r="L66" s="1"/>
-      <c r="M66" s="1"/>
-      <c r="N66" s="1"/>
-      <c r="O66" s="1"/>
-      <c r="P66" s="1"/>
-      <c r="Q66" s="1"/>
+      <c r="J66" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="L66" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M66" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="N66" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O66" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="P66" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="Q66" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="R66" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S66" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T66" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U66" s="1"/>
       <c r="V66" s="1" t="s">
@@ -9326,55 +9326,41 @@
         <v>390</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="G67" s="1"/>
       <c r="H67" s="1" t="s">
         <v>391</v>
       </c>
       <c r="I67" s="1"/>
-      <c r="J67" s="1" t="s">
-        <v>392</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="L67" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="M67" s="1" t="s">
-        <v>390</v>
-      </c>
-      <c r="N67" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O67" s="1" t="s">
-        <v>394</v>
-      </c>
+      <c r="J67" s="1"/>
+      <c r="K67" s="1"/>
+      <c r="L67" s="1"/>
+      <c r="M67" s="1"/>
+      <c r="N67" s="1"/>
+      <c r="O67" s="1"/>
       <c r="P67" s="1"/>
-      <c r="Q67" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="Q67" s="1"/>
       <c r="R67" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S67" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T67" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U67" s="1"/>
       <c r="V67" s="1" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
     <row r="68" spans="1:22">
       <c r="A68" s="1" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="B68" s="1">
         <v>31447154</v>
@@ -9386,32 +9372,46 @@
         <v>390</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="G68" s="1"/>
       <c r="H68" s="1" t="s">
         <v>391</v>
       </c>
       <c r="I68" s="1"/>
-      <c r="J68" s="1"/>
-      <c r="K68" s="1"/>
-      <c r="L68" s="1"/>
-      <c r="M68" s="1"/>
-      <c r="N68" s="1"/>
-      <c r="O68" s="1"/>
+      <c r="J68" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="K68" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="L68" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="M68" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="N68" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O68" s="1" t="s">
+        <v>396</v>
+      </c>
       <c r="P68" s="1"/>
-      <c r="Q68" s="1"/>
+      <c r="Q68" s="1" t="s">
+        <v>38</v>
+      </c>
       <c r="R68" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S68" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T68" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U68" s="1"/>
       <c r="V68" s="1" t="s">
@@ -9440,31 +9440,43 @@
       <c r="G69" s="1"/>
       <c r="H69" s="1"/>
       <c r="I69" s="1"/>
-      <c r="J69" s="1"/>
-      <c r="K69" s="1"/>
+      <c r="J69" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="K69" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="L69" s="1"/>
-      <c r="M69" s="1"/>
-      <c r="N69" s="1"/>
-      <c r="O69" s="1"/>
+      <c r="M69" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="N69" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="O69" s="1" t="s">
+        <v>403</v>
+      </c>
       <c r="P69" s="1"/>
-      <c r="Q69" s="1"/>
+      <c r="Q69" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="R69" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S69" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T69" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U69" s="1"/>
       <c r="V69" s="1" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
     </row>
     <row r="70" spans="1:22">
       <c r="A70" s="1" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B70" s="1">
         <v>31455868</v>
@@ -9484,34 +9496,22 @@
       <c r="G70" s="1"/>
       <c r="H70" s="1"/>
       <c r="I70" s="1"/>
-      <c r="J70" s="1" t="s">
-        <v>403</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>361</v>
-      </c>
+      <c r="J70" s="1"/>
+      <c r="K70" s="1"/>
       <c r="L70" s="1"/>
-      <c r="M70" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="N70" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="O70" s="1" t="s">
-        <v>405</v>
-      </c>
+      <c r="M70" s="1"/>
+      <c r="N70" s="1"/>
+      <c r="O70" s="1"/>
       <c r="P70" s="1"/>
-      <c r="Q70" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="Q70" s="1"/>
       <c r="R70" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S70" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T70" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U70" s="1"/>
       <c r="V70" s="1" t="s">
@@ -9627,34 +9627,46 @@
       </c>
       <c r="G73" s="1"/>
       <c r="H73" s="1"/>
-      <c r="I73" s="1" t="s">
+      <c r="I73" s="1"/>
+      <c r="J73" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="J73" s="1"/>
-      <c r="K73" s="1"/>
-      <c r="L73" s="1"/>
-      <c r="M73" s="1"/>
-      <c r="N73" s="1"/>
-      <c r="O73" s="1"/>
+      <c r="K73" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="L73" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="M73" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="N73" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="O73" s="1" t="s">
+        <v>418</v>
+      </c>
       <c r="P73" s="1"/>
-      <c r="Q73" s="1"/>
+      <c r="Q73" s="1" t="s">
+        <v>38</v>
+      </c>
       <c r="R73" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S73" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T73" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U73" s="1"/>
       <c r="V73" s="1" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="74" spans="1:22">
       <c r="A74" s="1" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B74" s="1">
         <v>31475270</v>
@@ -9669,11 +9681,13 @@
         <v>26</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="G74" s="1"/>
       <c r="H74" s="1"/>
-      <c r="I74" s="1"/>
+      <c r="I74" s="1" t="s">
+        <v>422</v>
+      </c>
       <c r="J74" s="1"/>
       <c r="K74" s="1"/>
       <c r="L74" s="1"/>
@@ -9693,12 +9707,12 @@
       </c>
       <c r="U74" s="1"/>
       <c r="V74" s="1" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
     </row>
     <row r="75" spans="1:22">
       <c r="A75" s="1" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="B75" s="1">
         <v>31475270</v>
@@ -9713,41 +9727,27 @@
         <v>26</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="G75" s="1"/>
       <c r="H75" s="1"/>
       <c r="I75" s="1"/>
-      <c r="J75" s="1" t="s">
-        <v>423</v>
-      </c>
-      <c r="K75" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="L75" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="M75" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="N75" s="1" t="s">
-        <v>422</v>
-      </c>
-      <c r="O75" s="1" t="s">
-        <v>424</v>
-      </c>
+      <c r="J75" s="1"/>
+      <c r="K75" s="1"/>
+      <c r="L75" s="1"/>
+      <c r="M75" s="1"/>
+      <c r="N75" s="1"/>
+      <c r="O75" s="1"/>
       <c r="P75" s="1"/>
-      <c r="Q75" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="Q75" s="1"/>
       <c r="R75" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S75" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T75" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U75" s="1"/>
       <c r="V75" s="1" t="s">
@@ -9766,39 +9766,53 @@
         <v>427</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="G76" s="1"/>
       <c r="H76" s="1"/>
       <c r="I76" s="1"/>
-      <c r="J76" s="1"/>
-      <c r="K76" s="1"/>
+      <c r="J76" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="K76" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="L76" s="1"/>
-      <c r="M76" s="1"/>
-      <c r="N76" s="1"/>
-      <c r="O76" s="1"/>
-      <c r="P76" s="1"/>
-      <c r="Q76" s="1"/>
+      <c r="M76" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="N76" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O76" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="P76" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="Q76" s="1" t="s">
+        <v>80</v>
+      </c>
       <c r="R76" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S76" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T76" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U76" s="1"/>
       <c r="V76" s="1" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
     </row>
     <row r="77" spans="1:22">
       <c r="A77" s="1" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B77" s="1">
         <v>31485048</v>
@@ -9808,44 +9822,30 @@
         <v>427</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="G77" s="1"/>
       <c r="H77" s="1"/>
       <c r="I77" s="1"/>
-      <c r="J77" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="K77" s="1" t="s">
-        <v>361</v>
-      </c>
+      <c r="J77" s="1"/>
+      <c r="K77" s="1"/>
       <c r="L77" s="1"/>
-      <c r="M77" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="N77" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O77" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="P77" s="1" t="s">
-        <v>432</v>
-      </c>
-      <c r="Q77" s="1" t="s">
-        <v>80</v>
-      </c>
+      <c r="M77" s="1"/>
+      <c r="N77" s="1"/>
+      <c r="O77" s="1"/>
+      <c r="P77" s="1"/>
+      <c r="Q77" s="1"/>
       <c r="R77" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S77" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T77" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U77" s="1"/>
       <c r="V77" s="1" t="s">
@@ -10047,10 +10047,10 @@
         <v>453</v>
       </c>
       <c r="P81" s="1" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="Q81" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R81" s="1" t="s">
         <v>26</v>
@@ -10062,7 +10062,7 @@
         <v>29</v>
       </c>
       <c r="U81" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="V81" s="1" t="s">
         <v>454</v>
@@ -10082,39 +10082,49 @@
         <v>457</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="G82" s="1"/>
       <c r="H82" s="1"/>
       <c r="I82" s="1"/>
-      <c r="J82" s="1"/>
+      <c r="J82" s="1" t="s">
+        <v>456</v>
+      </c>
       <c r="K82" s="1"/>
       <c r="L82" s="1"/>
-      <c r="M82" s="1"/>
-      <c r="N82" s="1"/>
-      <c r="O82" s="1"/>
+      <c r="M82" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="N82" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O82" s="1" t="s">
+        <v>458</v>
+      </c>
       <c r="P82" s="1"/>
-      <c r="Q82" s="1"/>
+      <c r="Q82" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="R82" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S82" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T82" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U82" s="1"/>
       <c r="V82" s="1" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="83" spans="1:22">
       <c r="A83" s="1" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B83" s="1">
         <v>31544182</v>
@@ -10126,40 +10136,30 @@
         <v>457</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="G83" s="1"/>
       <c r="H83" s="1"/>
       <c r="I83" s="1"/>
-      <c r="J83" s="1" t="s">
-        <v>456</v>
-      </c>
+      <c r="J83" s="1"/>
       <c r="K83" s="1"/>
       <c r="L83" s="1"/>
-      <c r="M83" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="N83" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O83" s="1" t="s">
-        <v>460</v>
-      </c>
+      <c r="M83" s="1"/>
+      <c r="N83" s="1"/>
+      <c r="O83" s="1"/>
       <c r="P83" s="1"/>
-      <c r="Q83" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="Q83" s="1"/>
       <c r="R83" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S83" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T83" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U83" s="1"/>
       <c r="V83" s="1" t="s">
@@ -10282,39 +10282,53 @@
         <v>474</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="G86" s="1"/>
       <c r="H86" s="1"/>
       <c r="I86" s="1"/>
-      <c r="J86" s="1"/>
-      <c r="K86" s="1"/>
-      <c r="L86" s="1"/>
-      <c r="M86" s="1"/>
-      <c r="N86" s="1"/>
-      <c r="O86" s="1"/>
+      <c r="J86" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="K86" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="L86" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="M86" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="N86" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O86" s="1" t="s">
+        <v>477</v>
+      </c>
       <c r="P86" s="1"/>
-      <c r="Q86" s="1"/>
+      <c r="Q86" s="1" t="s">
+        <v>38</v>
+      </c>
       <c r="R86" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S86" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T86" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U86" s="1"/>
       <c r="V86" s="1" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="87" spans="1:22">
       <c r="A87" s="1" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B87" s="1">
         <v>31758865</v>
@@ -10326,44 +10340,30 @@
         <v>474</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="G87" s="1"/>
       <c r="H87" s="1"/>
       <c r="I87" s="1"/>
-      <c r="J87" s="1" t="s">
-        <v>477</v>
-      </c>
-      <c r="K87" s="1" t="s">
-        <v>361</v>
-      </c>
-      <c r="L87" s="1" t="s">
-        <v>478</v>
-      </c>
-      <c r="M87" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="N87" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O87" s="1" t="s">
-        <v>479</v>
-      </c>
+      <c r="J87" s="1"/>
+      <c r="K87" s="1"/>
+      <c r="L87" s="1"/>
+      <c r="M87" s="1"/>
+      <c r="N87" s="1"/>
+      <c r="O87" s="1"/>
       <c r="P87" s="1"/>
-      <c r="Q87" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="Q87" s="1"/>
       <c r="R87" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S87" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T87" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="U87" s="1"/>
       <c r="V87" s="1" t="s">
@@ -10401,7 +10401,7 @@
         <v>88</v>
       </c>
       <c r="L88" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="M88" s="1"/>
       <c r="N88" s="1" t="s">
@@ -10412,7 +10412,7 @@
       </c>
       <c r="P88" s="1"/>
       <c r="Q88" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R88" s="1" t="s">
         <v>26</v>
@@ -10594,7 +10594,7 @@
       </c>
       <c r="P91" s="1"/>
       <c r="Q91" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R91" s="1" t="s">
         <v>26</v>
@@ -10690,7 +10690,7 @@
       </c>
       <c r="P93" s="1"/>
       <c r="Q93" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R93" s="1" t="s">
         <v>29</v>
@@ -10746,7 +10746,7 @@
       </c>
       <c r="P94" s="1"/>
       <c r="Q94" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R94" s="1" t="s">
         <v>26</v>
@@ -10808,7 +10808,7 @@
       </c>
       <c r="P95" s="1"/>
       <c r="Q95" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R95" s="1" t="s">
         <v>26</v>
@@ -10864,7 +10864,7 @@
       </c>
       <c r="P96" s="1"/>
       <c r="Q96" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R96" s="1" t="s">
         <v>26</v>
@@ -10940,13 +10940,13 @@
         <v>33</v>
       </c>
       <c r="G98" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H98" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="I98" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="J98" s="1" t="s">
         <v>545</v>
@@ -10968,7 +10968,7 @@
       </c>
       <c r="P98" s="1"/>
       <c r="Q98" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R98" s="1" t="s">
         <v>26</v>
@@ -11022,7 +11022,7 @@
       </c>
       <c r="P99" s="1"/>
       <c r="Q99" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R99" s="1" t="s">
         <v>26</v>
@@ -11172,7 +11172,7 @@
         <v>571</v>
       </c>
       <c r="K102" s="1" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="L102" s="1" t="s">
         <v>111</v>
@@ -11188,7 +11188,7 @@
       </c>
       <c r="P102" s="1"/>
       <c r="Q102" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R102" s="1" t="s">
         <v>26</v>
@@ -11246,7 +11246,7 @@
       </c>
       <c r="P103" s="1"/>
       <c r="Q103" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R103" s="1" t="s">
         <v>26</v>
@@ -11298,7 +11298,7 @@
       </c>
       <c r="P104" s="1"/>
       <c r="Q104" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R104" s="1" t="s">
         <v>26</v>
@@ -11414,7 +11414,7 @@
       </c>
       <c r="P106" s="1"/>
       <c r="Q106" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R106" s="1" t="s">
         <v>26</v>
@@ -11470,7 +11470,7 @@
       </c>
       <c r="P107" s="1"/>
       <c r="Q107" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R107" s="1" t="s">
         <v>26</v>
@@ -11568,7 +11568,7 @@
       </c>
       <c r="P109" s="1"/>
       <c r="Q109" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R109" s="1" t="s">
         <v>29</v>
@@ -11600,7 +11600,7 @@
         <v>33</v>
       </c>
       <c r="G110" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H110" s="1"/>
       <c r="I110" s="1"/>
@@ -11654,10 +11654,10 @@
         <v>623</v>
       </c>
       <c r="K111" s="1" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="L111" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="M111" s="1"/>
       <c r="N111" s="1" t="s">
@@ -11764,7 +11764,7 @@
         <v>636</v>
       </c>
       <c r="I113" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="J113" s="1" t="s">
         <v>637</v>
@@ -12008,7 +12008,7 @@
         <v>665</v>
       </c>
       <c r="Q117" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R117" s="1" t="s">
         <v>26</v>
@@ -12126,7 +12126,7 @@
         <v>29</v>
       </c>
       <c r="U119" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="V119" s="1" t="s">
         <v>676</v>
@@ -12219,7 +12219,7 @@
         <v>88</v>
       </c>
       <c r="L121" s="1" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="M121" s="1" t="s">
         <v>686</v>
@@ -12277,7 +12277,7 @@
         <v>441</v>
       </c>
       <c r="L122" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="M122" s="1" t="s">
         <v>693</v>
@@ -12290,7 +12290,7 @@
       </c>
       <c r="P122" s="1"/>
       <c r="Q122" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R122" s="1" t="s">
         <v>26</v>
@@ -12396,7 +12396,7 @@
       </c>
       <c r="P124" s="1"/>
       <c r="Q124" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R124" s="1" t="s">
         <v>26</v>
@@ -12483,7 +12483,7 @@
         <v>88</v>
       </c>
       <c r="L126" s="1" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="M126" s="1" t="s">
         <v>710</v>
@@ -12496,7 +12496,7 @@
       </c>
       <c r="P126" s="1"/>
       <c r="Q126" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R126" s="1" t="s">
         <v>26</v>
@@ -12550,7 +12550,7 @@
       </c>
       <c r="P127" s="1"/>
       <c r="Q127" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R127" s="1" t="s">
         <v>26</v>
@@ -12726,7 +12726,7 @@
       </c>
       <c r="P130" s="1"/>
       <c r="Q130" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R130" s="1" t="s">
         <v>26</v>
@@ -12836,7 +12836,7 @@
         <v>754</v>
       </c>
       <c r="Q132" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R132" s="1" t="s">
         <v>26</v>
@@ -12898,7 +12898,7 @@
       </c>
       <c r="P133" s="1"/>
       <c r="Q133" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R133" s="1" t="s">
         <v>26</v>
@@ -12960,7 +12960,7 @@
       </c>
       <c r="P134" s="1"/>
       <c r="Q134" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R134" s="1" t="s">
         <v>26</v>
@@ -13020,7 +13020,7 @@
       </c>
       <c r="P135" s="1"/>
       <c r="Q135" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R135" s="1" t="s">
         <v>26</v>
@@ -13061,7 +13061,7 @@
         <v>321</v>
       </c>
       <c r="L136" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="M136" s="1" t="s">
         <v>779</v>
@@ -13074,7 +13074,7 @@
       </c>
       <c r="P136" s="1"/>
       <c r="Q136" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R136" s="1" t="s">
         <v>26</v>
@@ -13243,7 +13243,7 @@
         <v>26</v>
       </c>
       <c r="F140" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="G140" s="1"/>
       <c r="H140" s="1"/>
@@ -13261,7 +13261,7 @@
         <v>798</v>
       </c>
       <c r="N140" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="O140" s="1" t="s">
         <v>799</v>
@@ -13328,7 +13328,7 @@
       </c>
       <c r="P141" s="1"/>
       <c r="Q141" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R141" s="1" t="s">
         <v>26</v>
@@ -13442,7 +13442,7 @@
       </c>
       <c r="P143" s="1"/>
       <c r="Q143" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R143" s="1" t="s">
         <v>26</v>
@@ -13538,7 +13538,7 @@
       </c>
       <c r="P145" s="1"/>
       <c r="Q145" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R145" s="1" t="s">
         <v>26</v>
@@ -13636,7 +13636,7 @@
       </c>
       <c r="P147" s="1"/>
       <c r="Q147" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R147" s="1" t="s">
         <v>26</v>
@@ -13665,7 +13665,7 @@
         <v>26</v>
       </c>
       <c r="F148" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="G148" s="1"/>
       <c r="H148" s="1"/>
@@ -13683,7 +13683,7 @@
         <v>839</v>
       </c>
       <c r="N148" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="O148" s="1" t="s">
         <v>840</v>
@@ -13722,13 +13722,13 @@
         <v>33</v>
       </c>
       <c r="G149" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H149" s="1" t="s">
         <v>843</v>
       </c>
       <c r="I149" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="J149" s="1"/>
       <c r="K149" s="1"/>
@@ -13781,7 +13781,7 @@
         <v>321</v>
       </c>
       <c r="L150" s="1" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="M150" s="1"/>
       <c r="N150" s="1" t="s">
@@ -13792,7 +13792,7 @@
       </c>
       <c r="P150" s="1"/>
       <c r="Q150" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R150" s="1" t="s">
         <v>26</v>
@@ -13837,7 +13837,7 @@
         <v>321</v>
       </c>
       <c r="L151" s="1" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="M151" s="1" t="s">
         <v>854</v>
@@ -13850,7 +13850,7 @@
       </c>
       <c r="P151" s="1"/>
       <c r="Q151" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R151" s="1" t="s">
         <v>26</v>
@@ -13908,7 +13908,7 @@
       </c>
       <c r="P152" s="1"/>
       <c r="Q152" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R152" s="1" t="s">
         <v>26</v>
@@ -14075,7 +14075,7 @@
         <v>26</v>
       </c>
       <c r="F156" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="G156" s="1" t="s">
         <v>43</v>
@@ -14121,7 +14121,7 @@
         <v>26</v>
       </c>
       <c r="F157" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="G157" s="1"/>
       <c r="H157" s="1"/>
@@ -14184,7 +14184,7 @@
       </c>
       <c r="P158" s="1"/>
       <c r="Q158" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R158" s="1" t="s">
         <v>26</v>
@@ -14279,7 +14279,7 @@
         <v>321</v>
       </c>
       <c r="L160" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="M160" s="1" t="s">
         <v>888</v>
@@ -14331,10 +14331,10 @@
       </c>
       <c r="I161" s="1"/>
       <c r="J161" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K161" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="L161" s="1" t="s">
         <v>895</v>
@@ -14350,7 +14350,7 @@
       </c>
       <c r="P161" s="1"/>
       <c r="Q161" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R161" s="1" t="s">
         <v>26</v>
@@ -14390,7 +14390,7 @@
         <v>901</v>
       </c>
       <c r="K162" s="1" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="L162" s="1" t="s">
         <v>902</v>
@@ -14460,7 +14460,7 @@
       </c>
       <c r="P163" s="1"/>
       <c r="Q163" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R163" s="1" t="s">
         <v>26</v>
@@ -14502,7 +14502,7 @@
         <v>915</v>
       </c>
       <c r="K164" s="1" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="L164" s="1" t="s">
         <v>111</v>
@@ -14576,7 +14576,7 @@
       </c>
       <c r="P165" s="1"/>
       <c r="Q165" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R165" s="1" t="s">
         <v>26</v>
@@ -14632,7 +14632,7 @@
       </c>
       <c r="P166" s="1"/>
       <c r="Q166" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R166" s="1" t="s">
         <v>26</v>
@@ -14677,7 +14677,7 @@
         <v>110</v>
       </c>
       <c r="L167" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="M167" s="1" t="s">
         <v>931</v>
@@ -14721,7 +14721,7 @@
         <v>26</v>
       </c>
       <c r="F168" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="G168" s="1" t="s">
         <v>43</v>
@@ -14745,14 +14745,14 @@
         <v>937</v>
       </c>
       <c r="N168" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="O168" s="1" t="s">
         <v>941</v>
       </c>
       <c r="P168" s="1"/>
       <c r="Q168" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R168" s="1" t="s">
         <v>26</v>
@@ -14857,7 +14857,7 @@
         <v>321</v>
       </c>
       <c r="L170" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="M170" s="1" t="s">
         <v>952</v>
@@ -14961,7 +14961,7 @@
         <v>321</v>
       </c>
       <c r="L172" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="M172" s="1" t="s">
         <v>961</v>
@@ -15030,7 +15030,7 @@
       </c>
       <c r="P173" s="1"/>
       <c r="Q173" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R173" s="1" t="s">
         <v>26</v>
@@ -15059,7 +15059,7 @@
         <v>26</v>
       </c>
       <c r="F174" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="G174" s="1"/>
       <c r="H174" s="1"/>
@@ -15170,7 +15170,7 @@
       </c>
       <c r="P176" s="1"/>
       <c r="Q176" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R176" s="1" t="s">
         <v>26</v>
@@ -15211,7 +15211,7 @@
         <v>88</v>
       </c>
       <c r="L177" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="M177" s="1" t="s">
         <v>985</v>
@@ -15386,7 +15386,7 @@
       </c>
       <c r="P180" s="1"/>
       <c r="Q180" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R180" s="1" t="s">
         <v>26</v>
@@ -15444,7 +15444,7 @@
       </c>
       <c r="P181" s="1"/>
       <c r="Q181" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R181" s="1" t="s">
         <v>26</v>
@@ -15718,7 +15718,7 @@
       </c>
       <c r="P186" s="1"/>
       <c r="Q186" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R186" s="1" t="s">
         <v>26</v>
@@ -15778,7 +15778,7 @@
       </c>
       <c r="P187" s="1"/>
       <c r="Q187" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R187" s="1" t="s">
         <v>26</v>
@@ -15896,7 +15896,7 @@
       </c>
       <c r="P189" s="1"/>
       <c r="Q189" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R189" s="1" t="s">
         <v>26</v>
@@ -16206,7 +16206,7 @@
       </c>
       <c r="P195" s="1"/>
       <c r="Q195" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R195" s="1" t="s">
         <v>26</v>
@@ -16253,7 +16253,7 @@
         <v>88</v>
       </c>
       <c r="L196" s="1" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="M196" s="1" t="s">
         <v>312</v>
@@ -16266,7 +16266,7 @@
       </c>
       <c r="P196" s="1"/>
       <c r="Q196" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R196" s="1" t="s">
         <v>26</v>
@@ -16295,7 +16295,7 @@
         <v>26</v>
       </c>
       <c r="F197" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="G197" s="1"/>
       <c r="H197" s="1"/>
@@ -16307,11 +16307,11 @@
         <v>249</v>
       </c>
       <c r="L197" s="1" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="M197" s="1"/>
       <c r="N197" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="O197" s="1" t="s">
         <v>1098</v>
@@ -16440,7 +16440,7 @@
         <v>1114</v>
       </c>
       <c r="Q199" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R199" s="1" t="s">
         <v>26</v>
@@ -16558,7 +16558,7 @@
       </c>
       <c r="P201" s="1"/>
       <c r="Q201" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R201" s="1" t="s">
         <v>26</v>
@@ -16610,7 +16610,7 @@
       </c>
       <c r="P202" s="1"/>
       <c r="Q202" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R202" s="1" t="s">
         <v>26</v>
@@ -16659,7 +16659,7 @@
         <v>321</v>
       </c>
       <c r="L203" s="1" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="M203" s="1" t="s">
         <v>1138</v>
@@ -16672,7 +16672,7 @@
       </c>
       <c r="P203" s="1"/>
       <c r="Q203" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R203" s="1" t="s">
         <v>26</v>
@@ -16764,7 +16764,7 @@
         <v>1151</v>
       </c>
       <c r="K205" s="1" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="L205" s="1" t="s">
         <v>217</v>
@@ -16862,13 +16862,13 @@
         <v>33</v>
       </c>
       <c r="G207" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H207" s="1" t="s">
         <v>1160</v>
       </c>
       <c r="I207" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="J207" s="1"/>
       <c r="K207" s="1"/>
@@ -16936,7 +16936,7 @@
       </c>
       <c r="P208" s="1"/>
       <c r="Q208" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R208" s="1" t="s">
         <v>26</v>
@@ -16992,7 +16992,7 @@
       </c>
       <c r="P209" s="1"/>
       <c r="Q209" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R209" s="1" t="s">
         <v>26</v>
@@ -17054,7 +17054,7 @@
       </c>
       <c r="P210" s="1"/>
       <c r="Q210" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R210" s="1" t="s">
         <v>26</v>
@@ -17150,13 +17150,13 @@
         <v>33</v>
       </c>
       <c r="G212" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H212" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="I212" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="J212" s="1" t="s">
         <v>1195</v>
@@ -17269,7 +17269,7 @@
         <v>26</v>
       </c>
       <c r="F214" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="G214" s="1" t="s">
         <v>43</v>
@@ -17293,7 +17293,7 @@
         <v>1207</v>
       </c>
       <c r="N214" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="O214" s="1" t="s">
         <v>1208</v>
@@ -17441,7 +17441,7 @@
         <v>26</v>
       </c>
       <c r="F217" s="1" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="G217" s="1"/>
       <c r="H217" s="1"/>
@@ -17574,7 +17574,7 @@
       </c>
       <c r="P219" s="1"/>
       <c r="Q219" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R219" s="1" t="s">
         <v>26</v>
@@ -17668,13 +17668,13 @@
         <v>33</v>
       </c>
       <c r="G221" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H221" s="1" t="s">
         <v>1248</v>
       </c>
       <c r="I221" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="J221" s="1" t="s">
         <v>1249</v>
@@ -17698,7 +17698,7 @@
         <v>1252</v>
       </c>
       <c r="Q221" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R221" s="1" t="s">
         <v>26</v>
@@ -17780,7 +17780,7 @@
         <v>33</v>
       </c>
       <c r="G223" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H223" s="1" t="s">
         <v>1262</v>
@@ -17857,7 +17857,7 @@
         <v>522</v>
       </c>
       <c r="L224" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="M224" s="1" t="s">
         <v>1269</v>
@@ -18025,7 +18025,7 @@
         <v>1288</v>
       </c>
       <c r="L227" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="M227" s="1"/>
       <c r="N227" s="1" t="s">
@@ -18102,7 +18102,7 @@
         <v>1299</v>
       </c>
       <c r="Q228" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R228" s="1" t="s">
         <v>26</v>
@@ -18184,7 +18184,7 @@
         <v>1123</v>
       </c>
       <c r="G230" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H230" s="1"/>
       <c r="I230" s="1"/>
@@ -18253,7 +18253,7 @@
         <v>1288</v>
       </c>
       <c r="L231" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="M231" s="1" t="s">
         <v>1312</v>
@@ -18266,7 +18266,7 @@
       </c>
       <c r="P231" s="1"/>
       <c r="Q231" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R231" s="1" t="s">
         <v>26</v>
@@ -18313,7 +18313,7 @@
         <v>1288</v>
       </c>
       <c r="L232" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="M232" s="1" t="s">
         <v>1317</v>
@@ -18326,7 +18326,7 @@
       </c>
       <c r="P232" s="1"/>
       <c r="Q232" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R232" s="1" t="s">
         <v>26</v>
@@ -18398,7 +18398,7 @@
         <v>29</v>
       </c>
       <c r="U233" s="1" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="V233" s="1" t="s">
         <v>1329</v>
@@ -18578,7 +18578,7 @@
       </c>
       <c r="P236" s="1"/>
       <c r="Q236" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R236" s="1" t="s">
         <v>26</v>
@@ -18674,13 +18674,13 @@
         <v>33</v>
       </c>
       <c r="G238" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H238" s="1" t="s">
         <v>1357</v>
       </c>
       <c r="I238" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="J238" s="1" t="s">
         <v>1358</v>
@@ -18750,7 +18750,7 @@
         <v>1367</v>
       </c>
       <c r="K239" s="1" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="L239" s="1" t="s">
         <v>217</v>
@@ -18838,7 +18838,7 @@
         <v>29</v>
       </c>
       <c r="U240" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="V240" s="1" t="s">
         <v>1378</v>
@@ -18879,7 +18879,7 @@
         <v>1383</v>
       </c>
       <c r="L241" s="1" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="M241" s="1" t="s">
         <v>1384</v>
@@ -19200,7 +19200,7 @@
       </c>
       <c r="P246" s="1"/>
       <c r="Q246" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R246" s="1" t="s">
         <v>26</v>
@@ -19264,7 +19264,7 @@
       </c>
       <c r="P247" s="1"/>
       <c r="Q247" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R247" s="1" t="s">
         <v>26</v>
@@ -19328,7 +19328,7 @@
       </c>
       <c r="P248" s="1"/>
       <c r="Q248" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R248" s="1" t="s">
         <v>26</v>
@@ -19432,7 +19432,7 @@
         <v>1443</v>
       </c>
       <c r="K250" s="1" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="L250" s="1" t="s">
         <v>639</v>
@@ -19508,7 +19508,7 @@
       </c>
       <c r="P251" s="1"/>
       <c r="Q251" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R251" s="1" t="s">
         <v>26</v>
@@ -19544,13 +19544,13 @@
         <v>33</v>
       </c>
       <c r="G252" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H252" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="I252" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="J252" s="1" t="s">
         <v>1450</v>
@@ -19572,7 +19572,7 @@
       </c>
       <c r="P252" s="1"/>
       <c r="Q252" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R252" s="1" t="s">
         <v>26</v>
@@ -19685,7 +19685,7 @@
         <v>1471</v>
       </c>
       <c r="L254" s="1" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="M254" s="1" t="s">
         <v>1467</v>
@@ -19698,7 +19698,7 @@
       </c>
       <c r="P254" s="1"/>
       <c r="Q254" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R254" s="1" t="s">
         <v>26</v>
@@ -19758,7 +19758,7 @@
       </c>
       <c r="P255" s="1"/>
       <c r="Q255" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R255" s="1" t="s">
         <v>26</v>
@@ -19832,7 +19832,7 @@
         <v>29</v>
       </c>
       <c r="U256" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="V256" s="1" t="s">
         <v>1491</v>
@@ -19880,7 +19880,7 @@
       </c>
       <c r="P257" s="1"/>
       <c r="Q257" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R257" s="1" t="s">
         <v>26</v>
@@ -19938,7 +19938,7 @@
       </c>
       <c r="P258" s="1"/>
       <c r="Q258" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R258" s="1" t="s">
         <v>26</v>
@@ -19996,7 +19996,7 @@
       </c>
       <c r="P259" s="1"/>
       <c r="Q259" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R259" s="1" t="s">
         <v>26</v>
@@ -20056,7 +20056,7 @@
       </c>
       <c r="P260" s="1"/>
       <c r="Q260" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R260" s="1" t="s">
         <v>26</v>
@@ -20122,7 +20122,7 @@
       </c>
       <c r="P261" s="1"/>
       <c r="Q261" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R261" s="1" t="s">
         <v>26</v>
@@ -20306,7 +20306,7 @@
       </c>
       <c r="P264" s="1"/>
       <c r="Q264" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R264" s="1" t="s">
         <v>26</v>
@@ -20404,13 +20404,13 @@
         <v>33</v>
       </c>
       <c r="G266" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H266" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="I266" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="J266" s="1" t="s">
         <v>1560</v>
@@ -20483,7 +20483,7 @@
         <v>1571</v>
       </c>
       <c r="L267" s="1" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="M267" s="1" t="s">
         <v>1572</v>
@@ -20508,7 +20508,7 @@
         <v>29</v>
       </c>
       <c r="U267" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="V267" s="1" t="s">
         <v>1574</v>
@@ -20618,7 +20618,7 @@
       </c>
       <c r="P269" s="1"/>
       <c r="Q269" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R269" s="1" t="s">
         <v>26</v>
@@ -20662,10 +20662,10 @@
         <v>1586</v>
       </c>
       <c r="K270" s="1" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="L270" s="1" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="M270" s="1" t="s">
         <v>1584</v>
@@ -20750,7 +20750,7 @@
         <v>29</v>
       </c>
       <c r="U271" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="V271" s="1" t="s">
         <v>1599</v>
@@ -20789,7 +20789,7 @@
         <v>1375</v>
       </c>
       <c r="L272" s="1" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="M272" s="1" t="s">
         <v>1604</v>
@@ -20814,7 +20814,7 @@
         <v>29</v>
       </c>
       <c r="U272" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="V272" s="1" t="s">
         <v>1606</v>
@@ -20848,10 +20848,10 @@
         <v>1611</v>
       </c>
       <c r="K273" s="1" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="L273" s="1" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="M273" s="1" t="s">
         <v>1609</v>
@@ -20908,10 +20908,10 @@
         <v>1611</v>
       </c>
       <c r="K274" s="1" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="L274" s="1" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="M274" s="1" t="s">
         <v>1616</v>
@@ -21122,7 +21122,7 @@
         <v>29</v>
       </c>
       <c r="U277" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="V277" s="1" t="s">
         <v>1642</v>
@@ -21174,7 +21174,7 @@
       </c>
       <c r="P278" s="1"/>
       <c r="Q278" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R278" s="1" t="s">
         <v>26</v>
@@ -21236,7 +21236,7 @@
       </c>
       <c r="P279" s="1"/>
       <c r="Q279" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R279" s="1" t="s">
         <v>26</v>
@@ -21248,7 +21248,7 @@
         <v>29</v>
       </c>
       <c r="U279" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="V279" s="1" t="s">
         <v>1661</v>
@@ -21422,7 +21422,7 @@
         <v>29</v>
       </c>
       <c r="U282" s="1" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="V282" s="1" t="s">
         <v>1684</v>
@@ -21470,7 +21470,7 @@
       </c>
       <c r="P283" s="1"/>
       <c r="Q283" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R283" s="1" t="s">
         <v>26</v>
@@ -21519,7 +21519,7 @@
         <v>1696</v>
       </c>
       <c r="L284" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="M284" s="1" t="s">
         <v>1693</v>

</xml_diff>